<commit_message>
Updated TC4 and TC5 in LoginPage
</commit_message>
<xml_diff>
--- a/SauceDemoData.xlsx
+++ b/SauceDemoData.xlsx
@@ -4,18 +4,18 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Login Page Content"/>
-    <sheet r:id="rId2" sheetId="2" name="Login Page Data"/>
+    <sheet r:id="rId2" sheetId="2" name="Login Page TC Data"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>Test Case number</t>
   </si>
@@ -32,6 +32,9 @@
     <t>secret_sauce</t>
   </si>
   <si>
+    <t>secret_sauc</t>
+  </si>
+  <si>
     <t>Attribute</t>
   </si>
   <si>
@@ -65,10 +68,22 @@
     <t>rgb(61, 220, 145)</t>
   </si>
   <si>
-    <t>Error Message</t>
+    <t>Error Message 1</t>
   </si>
   <si>
     <t>Epic sadface: Username is required</t>
+  </si>
+  <si>
+    <t>Error Message 2</t>
+  </si>
+  <si>
+    <t>Epic sadface: Password is required</t>
+  </si>
+  <si>
+    <t>Error Message 3</t>
+  </si>
+  <si>
+    <t>Epic sadface: Username and password do not match any user in this service</t>
   </si>
 </sst>
 </file>
@@ -118,13 +133,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -434,67 +452,83 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="27.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="35.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="27.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="76.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -507,12 +541,12 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="21.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="25.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="27.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="21.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="25.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="27.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -527,14 +561,25 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1">
-        <v>2</v>
+      <c r="A2" s="3">
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>